<commit_message>
mise à jour fichier excel
</commit_message>
<xml_diff>
--- a/benchmark22.xlsx
+++ b/benchmark22.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\PA1PEPF000E8F78\EXCELCNV\71d6cf63-bfbf-4186-a35f-481255a6b4af\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A291960F-2CE6-4E9C-AE9E-DEC6EC092256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45623652-6F2F-487B-83C4-4A5ED16CE721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{9E2EE9B3-0B78-4B65-9782-A1E9BFEFD141}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="60">
   <si>
     <t>objective gurobi</t>
   </si>
@@ -56,6 +56,15 @@
     <t>Solve time</t>
   </si>
   <si>
+    <t>objective CCopt</t>
+  </si>
+  <si>
+    <t>Status CCopt</t>
+  </si>
+  <si>
+    <t>Solve time CCopt</t>
+  </si>
+  <si>
     <t>risky_investment</t>
   </si>
   <si>
@@ -68,6 +77,9 @@
     <t>4.799000024795532</t>
   </si>
   <si>
+    <t>0.3100001811981201</t>
+  </si>
+  <si>
     <t>1d.jl</t>
   </si>
   <si>
@@ -77,6 +89,9 @@
     <t>27.990999937057495</t>
   </si>
   <si>
+    <t>282.15499997138977</t>
+  </si>
+  <si>
     <t>4d.jl</t>
   </si>
   <si>
@@ -86,6 +101,9 @@
     <t>6.224999904632568</t>
   </si>
   <si>
+    <t>20.575000047683716</t>
+  </si>
+  <si>
     <t>nodal_zonal_arbitrage_model</t>
   </si>
   <si>
@@ -95,6 +113,9 @@
     <t>0.11699986457824707</t>
   </si>
   <si>
+    <t>1.1659998893737793</t>
+  </si>
+  <si>
     <t>electricity_market_model</t>
   </si>
   <si>
@@ -104,6 +125,9 @@
     <t>0.012000083923339844</t>
   </si>
   <si>
+    <t>0.01699995994567871</t>
+  </si>
+  <si>
     <t>electric002_model</t>
   </si>
   <si>
@@ -113,6 +137,9 @@
     <t>0.8849999904632568</t>
   </si>
   <si>
+    <t>0.192000150680542</t>
+  </si>
+  <si>
     <t>electric004_model</t>
   </si>
   <si>
@@ -122,6 +149,9 @@
     <t>2.0480000972747803</t>
   </si>
   <si>
+    <t>6.388999938964844</t>
+  </si>
+  <si>
     <t>ex001_epec_model</t>
   </si>
   <si>
@@ -134,6 +164,9 @@
     <t>0.009000062942504883</t>
   </si>
   <si>
+    <t>-4.647622032433908e-9</t>
+  </si>
+  <si>
     <t>ex4_epec_model</t>
   </si>
   <si>
@@ -149,6 +182,9 @@
     <t>0.3509998321533203</t>
   </si>
   <si>
+    <t>0.44899988174438477</t>
+  </si>
+  <si>
     <t>outrata3_epec_model</t>
   </si>
   <si>
@@ -161,6 +197,9 @@
     <t>2.1519999504089355</t>
   </si>
   <si>
+    <t>1.9350001811981201</t>
+  </si>
+  <si>
     <t>outrata4_epec_model</t>
   </si>
   <si>
@@ -173,7 +212,7 @@
     <t>37.1425135255005</t>
   </si>
   <si>
-    <t>0.01699995994567871</t>
+    <t>0.04999995231628418</t>
   </si>
   <si>
     <t>market_power.jl</t>
@@ -1017,10 +1056,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40108776-88D3-447B-A13B-1D0BD658821B}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:11">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1039,296 +1078,371 @@
       <c r="G1" t="s">
         <v>5</v>
       </c>
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="13.5" customHeight="1">
+    <row r="2" spans="1:11" ht="13.5" customHeight="1">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="I6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="I9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
+        <v>47</v>
+      </c>
+      <c r="I10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
+        <v>52</v>
+      </c>
+      <c r="I11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="I12" t="s">
+        <v>10</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1348,8 +1462,25 @@
       <c r="G13">
         <v>7.4570000171661297</v>
       </c>
-      <c r="H13">
-        <v>0</v>
+      <c r="I13" t="s">
+        <v>10</v>
+      </c>
+      <c r="J13" t="s">
+        <v>10</v>
+      </c>
+      <c r="K13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="I14" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" t="s">
+        <v>10</v>
+      </c>
+      <c r="K14" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>